<commit_message>
Cleaned up everything; should be ready to submit!
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\hack-club\chord-board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAD6CE9-3372-4AD1-85EF-87CB121D25B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4577BE1-E7FA-406E-A2ED-1C3E99486959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{20DA92CE-7898-4CA1-90AB-3ECA5FA23D91}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="107">
   <si>
     <t>Part</t>
   </si>
@@ -258,6 +258,108 @@
   </si>
   <si>
     <t>250g filament for case (299.20467012cm^3 needed)</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/cherry-americas-llc/MX2A-51NB/21738393</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/bourns-inc/PTV09A-4020U-B103/3781130</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/bourns-inc/PTL45-15O0-105A2/3781312</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/dfrobot/DFR0847/15848097</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/cw-industries/GPTS203211B/3190590</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/adafruit-industries-llc/4960/14302512</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/mcc-micro-commercial-components/1N4148W-TP/717196</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/seeed-technology-co-ltd/113991054/16652880</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/CD74HC4067M96/1507236</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-0710KL/726880</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/evvo/1N5819W/21407174</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/c-k/S201031MS02Q/2055169</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/bourns-inc/CR0603-FX-5100ELF/3784063</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/pui-audio-inc/SMS-1804MS-HT/22116413</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/laird-signal-integrity-products/MI0603L301R-10/806613</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/diodes-incorporated/PAM8403DR-H/4033372</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/bourns-inc/PTV112-4420A-A103/3780862</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B104KB8NNNC/3886658</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/kemet/C0603C221K1RACTU/2200223</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B474KO8NNNC/3886720</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B105KO8NNNC/3886677</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM21BZ71A226ME15L/13904953</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21A476MRYNNNE/3888577</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRM21BR60G107ME11L/6155750</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/keystone-electronics/1043P/4499388</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/toshiba-semiconductor-and-storage/74HC595D/5879984</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/adafruit-industries-llc/6250/26249971</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/zeus-battery-products/PCIFR18650-1500/9828824</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/2255799834652852.html?spm=a2g0o.productlist.main.37.6b874ed6BcWYjZ&amp;algo_pvid=cd074ac6-6a57-4cf5-981a-391588099b78&amp;algo_exp_id=cd074ac6-6a57-4cf5-981a-391588099b78-26&amp;pdp_ext_f=%7B%22order%22%3A%222600%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%211.88%211.14%21%21%211.88%211.14%21%402101e2b617816772954112557ea7ef%2110000000048589927%21sea%21US%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3A1810974d%3Bm03_new_user%3A-29895%3BpisId%3A5000000208023469&amp;curPageLogUid=YDdz2iuLNXm6&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A4000020967604%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256808711257006.html?spm=a2g0o.productlist.main.2.588712795JXjaS&amp;algo_pvid=3b7e86bf-95d4-4a1f-8bfc-446c23c8ca52&amp;algo_exp_id=3b7e86bf-95d4-4a1f-8bfc-446c23c8ca52-1&amp;pdp_ext_f=%7B%22order%22%3A%2214336%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%212.04%210.99%21%21%2113.73%216.65%21%4021032f3717816763074298747ec926%2112000047114716314%21sea%21US%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3A1810974d%3Bm03_new_user%3A-29895%3BpisId%3A5000000207262921&amp;curPageLogUid=6LOCmPzaGrDu&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005008897571758%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/2255800276960438.html?spm=a2g0o.productlist.main.1.29b6HGVqHGVqk9&amp;algo_pvid=f62fd8ef-89c5-4cec-9183-177d8f962862&amp;algo_exp_id=f62fd8ef-89c5-4cec-9183-177d8f962862-0&amp;pdp_ext_f=%7B%22order%22%3A%22180%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%211.16%210.99%21%21%211.16%210.99%21%402101d97817816783189382683e3d6f%2112000016614368200%21sea%21US%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3A1810974d%3Bm03_new_user%3A-29895%3BpisId%3A5000000208023469&amp;curPageLogUid=hPayhJG0pxXX&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A4000463275190%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256806976696840.html?spm=a2g0o.productlist.main.2.1c33cd0fZpruBy&amp;algo_pvid=19866c55-1e6a-443f-a7a9-0dd49705db3d&amp;algo_exp_id=19866c55-1e6a-443f-a7a9-0dd49705db3d-34&amp;pdp_ext_f=%7B%22order%22%3A%22359%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%216.34%210.99%21%21%216.34%210.99%21%402101e83017819059640583970e0300%2112000039662452078%21sea%21US%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Adcd69f6e%3Bm03_new_user%3A-29895%3BpisId%3A5000000207262921&amp;curPageLogUid=lXV8t9sE9sV8&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005007163011592%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>Total Cost:</t>
   </si>
 </sst>
 </file>
@@ -640,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77098CAA-D477-4129-999C-610E4ADC381C}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.81640625" customWidth="1"/>
@@ -649,692 +751,811 @@
     <col min="5" max="5" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>9</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>1.75</v>
       </c>
-      <c r="E2">
-        <f>D2*C2</f>
+      <c r="F2">
+        <f>E2*D2</f>
         <v>15.75</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" t="s">
         <v>24</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>7</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>0.89</v>
       </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E36" si="0">D3*C3</f>
+      <c r="F3">
+        <f t="shared" ref="F3:F36" si="0">E3*D3</f>
         <v>6.23</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
       <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
         <v>2.57</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <f t="shared" si="0"/>
         <v>2.57</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
       <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
         <v>8.9</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <f t="shared" si="0"/>
         <v>8.9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>2</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>1.94</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <f t="shared" si="0"/>
         <v>3.88</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>4960</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
         <v>22</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>9</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>2.95</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <f t="shared" si="0"/>
         <v>26.55</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" t="s">
         <v>10</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>10</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>6.3E-2</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <f t="shared" si="0"/>
         <v>0.63</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" t="s">
         <v>5</v>
       </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
       <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <v>4.99</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <f t="shared" si="0"/>
         <v>4.99</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" t="s">
         <v>7</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
       <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
         <v>0.89</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <f t="shared" si="0"/>
         <v>0.89</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" t="s">
         <v>38</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>10</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" t="s">
         <v>12</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>2</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>0.23</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <f t="shared" si="0"/>
         <v>0.46</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" t="s">
         <v>14</v>
       </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
       <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
         <v>5.86</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <f t="shared" si="0"/>
         <v>5.86</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" t="s">
         <v>39</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>2</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>0.1</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" t="s">
         <v>29</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>2</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>4.8600000000000003</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <f t="shared" si="0"/>
         <v>9.7200000000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" t="s">
         <v>31</v>
       </c>
-      <c r="C16">
+      <c r="D16">
         <v>4</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>0.1</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" t="s">
         <v>33</v>
       </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
       <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
         <v>0.8</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <f t="shared" si="0"/>
         <v>0.8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
       <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
         <v>1.65</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <f t="shared" si="0"/>
         <v>1.65</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" t="s">
         <v>37</v>
       </c>
-      <c r="C19">
+      <c r="D19">
         <v>10</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>2.7E-2</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <f t="shared" si="0"/>
         <v>0.27</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" t="s">
         <v>41</v>
       </c>
-      <c r="C20">
+      <c r="D20">
         <v>4</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>0.1</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" t="s">
         <v>44</v>
       </c>
-      <c r="C21">
+      <c r="D21">
         <v>2</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>0.1</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" t="s">
         <v>45</v>
       </c>
-      <c r="C22">
+      <c r="D22">
         <v>10</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <f t="shared" si="0"/>
         <v>0.37</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" t="s">
         <v>47</v>
       </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
       <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
         <v>0.33</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <f t="shared" si="0"/>
         <v>0.33</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C24" t="s">
         <v>49</v>
       </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
       <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24">
         <v>0.26</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <f t="shared" si="0"/>
         <v>0.26</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" t="s">
         <v>51</v>
       </c>
-      <c r="C25">
+      <c r="D25">
         <v>4</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>0.55000000000000004</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <f t="shared" si="0"/>
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" t="s">
         <v>53</v>
       </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
       <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
         <v>3.02</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <f t="shared" si="0"/>
         <v>3.02</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" t="s">
         <v>55</v>
       </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
       <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
         <v>0.27</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <f t="shared" si="0"/>
         <v>0.27</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>6250</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" t="s">
         <v>56</v>
       </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
       <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
         <v>4.95</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <f t="shared" si="0"/>
         <v>4.95</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" t="s">
         <v>57</v>
       </c>
-      <c r="C29">
-        <v>1</v>
-      </c>
       <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
         <v>6.81</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <f t="shared" si="0"/>
         <v>6.81</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" t="s">
         <v>59</v>
       </c>
-      <c r="C30">
-        <v>1</v>
-      </c>
       <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30">
         <v>2.4900000000000002</v>
       </c>
-      <c r="E30">
+      <c r="F30">
         <f t="shared" si="0"/>
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" t="s">
         <v>62</v>
       </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
       <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31">
         <v>2.0099999999999998</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <f t="shared" si="0"/>
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" t="s">
         <v>64</v>
       </c>
-      <c r="C32">
-        <v>1</v>
-      </c>
       <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
         <v>2.63</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <f t="shared" si="0"/>
         <v>2.63</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" t="s">
         <v>66</v>
       </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
       <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="E33">
         <v>2.13</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <f t="shared" si="0"/>
         <v>2.13</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" t="s">
         <v>68</v>
       </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
       <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
         <v>1.1599999999999999</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <f t="shared" si="0"/>
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" t="s">
         <v>70</v>
       </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
       <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
         <v>1.23</v>
       </c>
-      <c r="E35">
+      <c r="F35">
         <f t="shared" si="0"/>
         <v>1.23</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" t="s">
         <v>72</v>
       </c>
-      <c r="C36">
-        <v>1</v>
-      </c>
       <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
         <v>11.46</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <f t="shared" si="0"/>
         <v>11.46</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E37" t="s">
+        <v>106</v>
+      </c>
+      <c r="F37">
+        <f>SUM(F2:F36)</f>
+        <v>131.92000000000002</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="Cherry MX Key" xr:uid="{B961A2B6-A7B1-46CC-BC5A-705B55FDFE94}"/>
-    <hyperlink ref="A3" r:id="rId2" display="Linear Potentiometers" xr:uid="{DF7F1705-5A2B-46CC-B6B8-D2C5413649BD}"/>
-    <hyperlink ref="A4" r:id="rId3" display="Slide Potentiometers" xr:uid="{B541261C-9DCB-4133-BD3B-385A5A73AB1A}"/>
-    <hyperlink ref="A5" r:id="rId4" display="TFT Display" xr:uid="{9F9BD066-AB7E-48B4-9C90-437066656DE1}"/>
-    <hyperlink ref="A6" r:id="rId5" display="Latching Button" xr:uid="{A89B5F3A-B35F-4F60-A7A4-0E0C7DE1AADA}"/>
-    <hyperlink ref="A7" r:id="rId6" display="Reverse Mount LEDs" xr:uid="{B76A657C-605B-4D7A-9E2E-AB87A93528BE}"/>
-    <hyperlink ref="A8" r:id="rId7" display="1N4148W-TP Diodes" xr:uid="{FAB0910B-BF24-45E5-AC64-55BB19E943BC}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{0FF1DE24-F24B-4FED-89DF-151093D39B30}"/>
-    <hyperlink ref="A10" r:id="rId9" xr:uid="{D5F0014C-FDA5-4EE6-9D92-E172F4F96554}"/>
-    <hyperlink ref="A11" r:id="rId10" xr:uid="{5EB5024B-8C90-46F7-89F1-F336392CF349}"/>
-    <hyperlink ref="A12" r:id="rId11" xr:uid="{289BB4B9-AF25-4498-ACDF-9C332CF3AD67}"/>
-    <hyperlink ref="A13" r:id="rId12" display="On-Off Switch" xr:uid="{DCE61170-09C2-4FDB-A20A-7782F60F42B8}"/>
-    <hyperlink ref="A14" r:id="rId13" xr:uid="{95C2D00E-D778-4739-97DE-19C5C9767F42}"/>
-    <hyperlink ref="A15" r:id="rId14" xr:uid="{AF3DFEA7-8ED0-4713-BC64-E80CD63AE4BA}"/>
-    <hyperlink ref="A16" r:id="rId15" xr:uid="{6C51CD0C-DCDA-4E94-9190-AC25905BDB05}"/>
-    <hyperlink ref="A17" r:id="rId16" xr:uid="{A056EA46-1A97-4917-B449-EFE5E2BDCFAB}"/>
-    <hyperlink ref="A18" r:id="rId17" display="https://www.digikey.com/en/products/detail/bourns-inc/PTV112-4420A-A103/3780862" xr:uid="{7ED28C11-C788-4F68-8E2D-F73ED8EF6A4F}"/>
-    <hyperlink ref="A19" r:id="rId18" display="https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B104KB8NNNC/3886658" xr:uid="{96758F11-D369-40F2-818A-10032BF10666}"/>
-    <hyperlink ref="A20" r:id="rId19" display="https://www.digikey.com/en/products/detail/kemet/C0603C221K1RACTU/2200223" xr:uid="{5B9D6DE1-8A52-4F43-81B4-9597D31BC9A1}"/>
-    <hyperlink ref="A21" r:id="rId20" display="https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B474KO8NNNC/3886720" xr:uid="{E08182AD-C14F-4C6E-863D-B8795F7668BB}"/>
-    <hyperlink ref="A22" r:id="rId21" display="https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL10B105KO8NNNC/3886677" xr:uid="{C282CDCF-A050-4F22-BAD2-62DCC189E03F}"/>
-    <hyperlink ref="A23" r:id="rId22" display="https://www.digikey.com/en/products/detail/murata-electronics/GRM21BZ71A226ME15L/13904953" xr:uid="{BE24D35C-7F77-47EA-8156-8074FEEDACAD}"/>
-    <hyperlink ref="A24" r:id="rId23" display="https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21A476MRYNNNE/3888577" xr:uid="{A2B84EE5-F171-4209-9847-DEEB9DED5B20}"/>
-    <hyperlink ref="A25" r:id="rId24" display="https://www.digikey.com/en/products/detail/murata-electronics/GRM21BR60G107ME11L/6155750" xr:uid="{4FF5D216-8D54-4B3E-98AF-D6027F425E57}"/>
-    <hyperlink ref="A26" r:id="rId25" display="https://www.digikey.com/en/products/detail/keystone-electronics/1043P/4499388" xr:uid="{0EC9BDEE-C794-4AE8-8B9D-BBFB2B10E8A4}"/>
-    <hyperlink ref="A27" r:id="rId26" display="https://www.digikey.com/en/products/detail/toshiba-semiconductor-and-storage/74HC595D/5879984" xr:uid="{C25E909E-76D9-4682-AE9C-1BE1775A7DAC}"/>
-    <hyperlink ref="A28" r:id="rId27" display="https://www.digikey.com/en/products/detail/adafruit-industries-llc/6250/26249971" xr:uid="{0B66E8F1-7732-4DCE-8AF0-32C784A7E0FA}"/>
-    <hyperlink ref="A29" r:id="rId28" display="https://www.digikey.com/en/products/detail/zeus-battery-products/PCIFR18650-1500/9828824" xr:uid="{FA3ECFC5-13A6-479C-BC0E-8B8F30D5332E}"/>
-    <hyperlink ref="A30" r:id="rId29" display="M3 12mm Screws" xr:uid="{C97AFB88-3346-4088-B8BC-7D958A11CA30}"/>
-    <hyperlink ref="A31" r:id="rId30" xr:uid="{C9A9612B-C838-4AEA-99CA-B1E1C18A9971}"/>
-    <hyperlink ref="A32" r:id="rId31" xr:uid="{CDBB6071-B2A0-42AD-8331-5E0D42B9AB8D}"/>
-    <hyperlink ref="A33" r:id="rId32" xr:uid="{A5ABAD83-00A1-4BFF-897B-9D29F0836104}"/>
-    <hyperlink ref="A34" r:id="rId33" xr:uid="{21CB0502-FBCC-4EF8-9C98-D52D44AB4A12}"/>
-    <hyperlink ref="A35" r:id="rId34" xr:uid="{32D44385-BD3D-4767-ADAE-78CED4AD1884}"/>
-    <hyperlink ref="A36" r:id="rId35" display="Black PLA FIlament" xr:uid="{59F6BD33-3975-4231-8E9D-0FAE5ABF52B9}"/>
+    <hyperlink ref="A2" r:id="rId1" display="Cherry MX Key" xr:uid="{354508CB-4981-45B9-8D60-A0BF039F07B8}"/>
+    <hyperlink ref="A3" r:id="rId2" xr:uid="{C689D467-FBA5-4EB6-A6BB-5AB270B239F8}"/>
+    <hyperlink ref="A4" r:id="rId3" display="Slide Potentiometers" xr:uid="{0E5141DF-C74B-40B7-A008-46A5AFCBD215}"/>
+    <hyperlink ref="A5" r:id="rId4" xr:uid="{FEF28CD2-3AA6-461F-9ECB-3EAA00E61442}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{B964F7ED-06BE-4C85-888C-49415B8D7244}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.digikey.com/en/products/detail/adafruit-industries-llc/4960/14302512" xr:uid="{C27FC503-6A5A-4848-8357-08C7BE6FE222}"/>
+    <hyperlink ref="A8" r:id="rId7" xr:uid="{057C30EC-D6A9-44A1-BE4A-7EE5FF15B8E8}"/>
+    <hyperlink ref="A9" r:id="rId8" xr:uid="{81E30B67-DBB8-4038-BC0D-6B3CDE8CB290}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{24ED2D0F-BEC1-4160-BB17-19A17B16E771}"/>
+    <hyperlink ref="A11" r:id="rId10" xr:uid="{8225BA7C-CBE1-42CC-A800-01E755161934}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{F7C6CBD8-4EC9-4BF2-B3F2-AD041EC4D327}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{AE23C050-43A4-46FD-BFA3-D17A96A53A5C}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{56B0B85E-DEBF-4D49-97D7-B1F6BF73ED96}"/>
+    <hyperlink ref="A15" r:id="rId14" xr:uid="{ED2DB607-B70E-4AE5-8945-06364D684DD8}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{F23463C1-E128-4F85-BB2C-E8398AC4C597}"/>
+    <hyperlink ref="A17" r:id="rId16" xr:uid="{5D64DFAA-1122-4F12-8DBE-06C791C67603}"/>
+    <hyperlink ref="A18" r:id="rId17" xr:uid="{4A8BDCA0-F9D4-47F6-9F1A-1D6C374ADDF9}"/>
+    <hyperlink ref="A19" r:id="rId18" xr:uid="{3537BA13-E916-4FB8-9CBC-8EBBE484332A}"/>
+    <hyperlink ref="A20" r:id="rId19" xr:uid="{7DD4D0BD-FAB1-4F58-B023-393F9888FD98}"/>
+    <hyperlink ref="A21" r:id="rId20" xr:uid="{D70AAA36-52F6-4C44-8D35-D634A9EFDE9C}"/>
+    <hyperlink ref="A22" r:id="rId21" xr:uid="{D641A998-A443-45F8-85A5-49C78BDDC8E0}"/>
+    <hyperlink ref="A23" r:id="rId22" xr:uid="{D49DF488-6813-4E52-A7F3-8A1721D8B509}"/>
+    <hyperlink ref="A24" r:id="rId23" xr:uid="{82704705-94B2-4832-8362-F902DCB4537B}"/>
+    <hyperlink ref="A25" r:id="rId24" xr:uid="{B2A279FC-FD15-4748-98D4-0F85763DD07E}"/>
+    <hyperlink ref="A26" r:id="rId25" xr:uid="{A53B70F0-7A2A-4FBF-A5E1-8D90FA755B74}"/>
+    <hyperlink ref="A27" r:id="rId26" xr:uid="{86238364-BF9B-44D8-81E0-4C83946FE5D4}"/>
+    <hyperlink ref="A28" r:id="rId27" display="https://www.digikey.com/en/products/detail/adafruit-industries-llc/6250/26249971" xr:uid="{6E00F3B1-266B-4F45-93AB-D1A15E3126E5}"/>
+    <hyperlink ref="A29" r:id="rId28" xr:uid="{56E83D99-1910-415C-BA3C-70336EE376A7}"/>
+    <hyperlink ref="A30" r:id="rId29" xr:uid="{5A8248DD-E510-420A-9900-DF314AF51FAE}"/>
+    <hyperlink ref="A31" r:id="rId30" xr:uid="{A79BD419-F311-465B-A41B-4635CD51327B}"/>
+    <hyperlink ref="A32" r:id="rId31" xr:uid="{32D12244-990D-4A5B-A4E2-8ABD422F538B}"/>
+    <hyperlink ref="A33" r:id="rId32" xr:uid="{B04B1EF3-440C-4ED0-81BC-9A5889DB901F}"/>
+    <hyperlink ref="A34" r:id="rId33" xr:uid="{2EBF4920-7444-4B89-8EB9-AA27CF6D6149}"/>
+    <hyperlink ref="A35" r:id="rId34" xr:uid="{402E6B92-C04C-4614-829A-02823CF98735}"/>
+    <hyperlink ref="A36" r:id="rId35" xr:uid="{A2586B19-2BED-494D-8AD2-9489865D81BB}"/>
+    <hyperlink ref="B4" r:id="rId36" xr:uid="{DB5FECDB-4169-48E6-84DA-E1A6016B7F71}"/>
+    <hyperlink ref="B21" r:id="rId37" xr:uid="{4C8EF23C-4FE3-4D57-994C-D9C28F8C7886}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId36"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId38"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added firmware instructions to README, PCB price to BOM, and removed boundaries from Zine
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\hack-club\chord-board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4577BE1-E7FA-406E-A2ED-1C3E99486959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3ACFF17-50D6-420B-B4F3-A6D17090660A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{20DA92CE-7898-4CA1-90AB-3ECA5FA23D91}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="111">
   <si>
     <t>Part</t>
   </si>
@@ -360,6 +360,18 @@
   </si>
   <si>
     <t>Total Cost:</t>
+  </si>
+  <si>
+    <t>PCB Price</t>
+  </si>
+  <si>
+    <t>PCB Shipping</t>
+  </si>
+  <si>
+    <t>JLCPCB</t>
+  </si>
+  <si>
+    <t>Global standard direct line</t>
   </si>
 </sst>
 </file>
@@ -742,12 +754,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77098CAA-D477-4129-999C-610E4ADC381C}">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.81640625" customWidth="1"/>
-    <col min="2" max="2" width="37.54296875" customWidth="1"/>
-    <col min="3" max="4" width="21.36328125" customWidth="1"/>
+    <col min="2" max="2" width="89.90625" customWidth="1"/>
+    <col min="3" max="3" width="43.54296875" customWidth="1"/>
+    <col min="4" max="4" width="21.36328125" customWidth="1"/>
     <col min="5" max="5" width="17.453125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -809,7 +822,7 @@
         <v>0.89</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F36" si="0">E3*D3</f>
+        <f t="shared" ref="F3:F38" si="0">E3*D3</f>
         <v>6.23</v>
       </c>
     </row>
@@ -1507,12 +1520,48 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="E37" t="s">
+      <c r="A37" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" t="s">
+        <v>109</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>13.5</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="0"/>
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>108</v>
+      </c>
+      <c r="C38" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>12</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="E39" t="s">
         <v>106</v>
       </c>
-      <c r="F37">
-        <f>SUM(F2:F36)</f>
-        <v>131.92000000000002</v>
+      <c r="F39">
+        <f>SUM(F2:F38)</f>
+        <v>157.42000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>